<commit_message>
test: improve operators, logical, math, text, lookup conformance fixtures
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/logical/boolean_logic.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/logical/boolean_logic.xlsx
@@ -20,27 +20,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t xml:space="preserve">id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">val</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t xml:space="preserve">a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b</t>
   </si>
   <si>
     <t xml:space="preserve">flag</t>
   </si>
   <si>
-    <t xml:space="preserve">and</t>
-  </si>
-  <si>
-    <t xml:space="preserve">or</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xor</t>
+    <t xml:space="preserve">and_ab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">or_ab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not_flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xor_ab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">and_gt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">or_gt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">true_fn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">false_fn</t>
   </si>
 </sst>
 </file>
@@ -317,7 +329,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -342,13 +354,25 @@
       <c r="G1" s="0" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="n">
         <v>10</v>
       </c>
       <c r="B2" s="0" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="C2" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -359,7 +383,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="b">
-        <f aca="false">OR(A2&gt;100,B2&gt;10)</f>
+        <f aca="false">OR(A2&gt;50,B2&gt;50)</f>
         <v>0</v>
       </c>
       <c r="F2" s="1" t="b">
@@ -367,16 +391,32 @@
         <v>0</v>
       </c>
       <c r="G2" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A2&gt;50,B2&gt;5)</f>
+        <f aca="false">_xlfn.XOR(A2&gt;0,B2&gt;0)</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="1" t="b">
+        <f aca="false">AND(A2&gt;10,A2&lt;100)</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="1" t="b">
+        <f aca="false">OR(A2=0,B2=0)</f>
+        <v>0</v>
+      </c>
+      <c r="J2" s="1" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="K2" s="1" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="B3" s="0" t="n">
-        <v>7.2</v>
+        <v>0</v>
       </c>
       <c r="C3" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -384,10 +424,10 @@
       </c>
       <c r="D3" s="1" t="b">
         <f aca="false">AND(A3&gt;0,B3&gt;0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" s="1" t="b">
-        <f aca="false">OR(A3&gt;100,B3&gt;10)</f>
+        <f aca="false">OR(A3&gt;50,B3&gt;50)</f>
         <v>0</v>
       </c>
       <c r="F3" s="1" t="b">
@@ -395,16 +435,32 @@
         <v>1</v>
       </c>
       <c r="G3" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A3&gt;50,B3&gt;5)</f>
-        <v>1</v>
+        <f aca="false">_xlfn.XOR(A3&gt;0,B3&gt;0)</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="1" t="b">
+        <f aca="false">AND(A3&gt;10,A3&lt;100)</f>
+        <v>0</v>
+      </c>
+      <c r="I3" s="1" t="b">
+        <f aca="false">OR(A3=0,B3=0)</f>
+        <v>1</v>
+      </c>
+      <c r="J3" s="1" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="K3" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="B4" s="0" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="C4" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -415,80 +471,128 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="b">
-        <f aca="false">OR(A4&gt;100,B4&gt;10)</f>
-        <v>0</v>
+        <f aca="false">OR(A4&gt;50,B4&gt;50)</f>
+        <v>1</v>
       </c>
       <c r="F4" s="1" t="b">
         <f aca="false">NOT(C4)</f>
         <v>0</v>
       </c>
       <c r="G4" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A4&gt;50,B4&gt;5)</f>
+        <f aca="false">_xlfn.XOR(A4&gt;0,B4&gt;0)</f>
+        <v>1</v>
+      </c>
+      <c r="H4" s="1" t="b">
+        <f aca="false">AND(A4&gt;10,A4&lt;100)</f>
+        <v>0</v>
+      </c>
+      <c r="I4" s="1" t="b">
+        <f aca="false">OR(A4=0,B4=0)</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="1" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="K4" s="1" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="n">
-        <v>100</v>
+        <v>-5</v>
       </c>
       <c r="B5" s="0" t="n">
-        <v>15.8</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="D5" s="1" t="b">
         <f aca="false">AND(A5&gt;0,B5&gt;0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="1" t="b">
-        <f aca="false">OR(A5&gt;100,B5&gt;10)</f>
-        <v>1</v>
+        <f aca="false">OR(A5&gt;50,B5&gt;50)</f>
+        <v>0</v>
       </c>
       <c r="F5" s="1" t="b">
         <f aca="false">NOT(C5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A5&gt;50,B5&gt;5)</f>
+        <f aca="false">_xlfn.XOR(A5&gt;0,B5&gt;0)</f>
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="b">
+        <f aca="false">AND(A5&gt;10,A5&lt;100)</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="1" t="b">
+        <f aca="false">OR(A5=0,B5=0)</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="1" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="K5" s="1" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="n">
-        <v>-5</v>
+        <v>50</v>
       </c>
       <c r="B6" s="0" t="n">
-        <v>-2.3</v>
+        <v>50</v>
       </c>
       <c r="C6" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="D6" s="1" t="b">
         <f aca="false">AND(A6&gt;0,B6&gt;0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="1" t="b">
-        <f aca="false">OR(A6&gt;100,B6&gt;10)</f>
+        <f aca="false">OR(A6&gt;50,B6&gt;50)</f>
         <v>0</v>
       </c>
       <c r="F6" s="1" t="b">
         <f aca="false">NOT(C6)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A6&gt;50,B6&gt;5)</f>
+        <f aca="false">_xlfn.XOR(A6&gt;0,B6&gt;0)</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="1" t="b">
+        <f aca="false">AND(A6&gt;10,A6&lt;100)</f>
+        <v>1</v>
+      </c>
+      <c r="I6" s="1" t="b">
+        <f aca="false">OR(A6=0,B6=0)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="1" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="K6" s="1" t="b">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="B7" s="0" t="n">
-        <v>8.1</v>
+        <v>0</v>
       </c>
       <c r="C7" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -496,10 +600,10 @@
       </c>
       <c r="D7" s="1" t="b">
         <f aca="false">AND(A7&gt;0,B7&gt;0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="1" t="b">
-        <f aca="false">OR(A7&gt;100,B7&gt;10)</f>
+        <f aca="false">OR(A7&gt;50,B7&gt;50)</f>
         <v>0</v>
       </c>
       <c r="F7" s="1" t="b">
@@ -507,16 +611,32 @@
         <v>1</v>
       </c>
       <c r="G7" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A7&gt;50,B7&gt;5)</f>
-        <v>1</v>
+        <f aca="false">_xlfn.XOR(A7&gt;0,B7&gt;0)</f>
+        <v>1</v>
+      </c>
+      <c r="H7" s="1" t="b">
+        <f aca="false">AND(A7&gt;10,A7&lt;100)</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="1" t="b">
+        <f aca="false">OR(A7=0,B7=0)</f>
+        <v>1</v>
+      </c>
+      <c r="J7" s="1" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="K7" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="B8" s="0" t="n">
-        <v>4.6</v>
+        <v>1</v>
       </c>
       <c r="C8" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -524,10 +644,10 @@
       </c>
       <c r="D8" s="1" t="b">
         <f aca="false">AND(A8&gt;0,B8&gt;0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="1" t="b">
-        <f aca="false">OR(A8&gt;100,B8&gt;10)</f>
+        <f aca="false">OR(A8&gt;50,B8&gt;50)</f>
         <v>0</v>
       </c>
       <c r="F8" s="1" t="b">
@@ -535,92 +655,68 @@
         <v>0</v>
       </c>
       <c r="G8" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A8&gt;50,B8&gt;5)</f>
-        <v>1</v>
+        <f aca="false">_xlfn.XOR(A8&gt;0,B8&gt;0)</f>
+        <v>1</v>
+      </c>
+      <c r="H8" s="1" t="b">
+        <f aca="false">AND(A8&gt;10,A8&lt;100)</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="1" t="b">
+        <f aca="false">OR(A8=0,B8=0)</f>
+        <v>1</v>
+      </c>
+      <c r="J8" s="1" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="K8" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="B9" s="0" t="n">
-        <v>0.5</v>
+        <v>99</v>
       </c>
       <c r="C9" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="D9" s="1" t="b">
         <f aca="false">AND(A9&gt;0,B9&gt;0)</f>
         <v>1</v>
       </c>
       <c r="E9" s="1" t="b">
-        <f aca="false">OR(A9&gt;100,B9&gt;10)</f>
-        <v>0</v>
+        <f aca="false">OR(A9&gt;50,B9&gt;50)</f>
+        <v>1</v>
       </c>
       <c r="F9" s="1" t="b">
         <f aca="false">NOT(C9)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A9&gt;50,B9&gt;5)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
-        <v>999</v>
-      </c>
-      <c r="B10" s="0" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="C10" s="1" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D10" s="1" t="b">
-        <f aca="false">AND(A10&gt;0,B10&gt;0)</f>
-        <v>1</v>
-      </c>
-      <c r="E10" s="1" t="b">
-        <f aca="false">OR(A10&gt;100,B10&gt;10)</f>
-        <v>1</v>
-      </c>
-      <c r="F10" s="1" t="b">
-        <f aca="false">NOT(C10)</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A10&gt;50,B10&gt;5)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
-        <v>42</v>
-      </c>
-      <c r="B11" s="0" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="C11" s="1" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D11" s="1" t="b">
-        <f aca="false">AND(A11&gt;0,B11&gt;0)</f>
-        <v>1</v>
-      </c>
-      <c r="E11" s="1" t="b">
-        <f aca="false">OR(A11&gt;100,B11&gt;10)</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="1" t="b">
-        <f aca="false">NOT(C11)</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="1" t="b">
-        <f aca="false">_xlfn.XOR(A11&gt;50,B11&gt;5)</f>
-        <v>1</v>
+        <f aca="false">_xlfn.XOR(A9&gt;0,B9&gt;0)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="1" t="b">
+        <f aca="false">AND(A9&gt;10,A9&lt;100)</f>
+        <v>1</v>
+      </c>
+      <c r="I9" s="1" t="b">
+        <f aca="false">OR(A9=0,B9=0)</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="1" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="K9" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>